<commit_message>
adaugare semnaturi in docs generate
</commit_message>
<xml_diff>
--- a/dist/Gestiune_clienti_sqlite_portabil_v3/_internal/mapping_tehnician.xlsx
+++ b/dist/Gestiune_clienti_sqlite_portabil_v3/_internal/mapping_tehnician.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Gestionare_clienti_cu SQLite\pythonProject1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA1B1F83-3322-40A5-8961-2D2C2DE20D48}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5965E363-BA63-419B-BD9D-9EE34C9799FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
   <si>
     <t>Sigiliu</t>
   </si>
@@ -46,6 +46,15 @@
   </si>
   <si>
     <t>SR044</t>
+  </si>
+  <si>
+    <t>Semnatura</t>
+  </si>
+  <si>
+    <t>grecu.png</t>
+  </si>
+  <si>
+    <t>semnaturi/pop.png</t>
   </si>
 </sst>
 </file>
@@ -363,13 +372,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="11.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>5</v>
       </c>
@@ -379,8 +390,11 @@
       <c r="C1" t="s">
         <v>4</v>
       </c>
+      <c r="D1" t="s">
+        <v>7</v>
+      </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -390,8 +404,11 @@
       <c r="C2">
         <v>236</v>
       </c>
+      <c r="D2" t="s">
+        <v>9</v>
+      </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -400,6 +417,9 @@
       </c>
       <c r="C3">
         <v>1817</v>
+      </c>
+      <c r="D3" t="s">
+        <v>8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>